<commit_message>
Actualizado: solo proveedores CABA + Bercomat
</commit_message>
<xml_diff>
--- a/presupuestos/comparativa_completa.xlsx
+++ b/presupuestos/comparativa_completa.xlsx
@@ -129,7 +129,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -151,11 +151,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -223,6 +267,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -682,16 +728,16 @@
           <t xml:space="preserve">  HOJA 1 — Revestimientos y Porcelanatos</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="B4" s="27" t="n"/>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="27" t="n"/>
+      <c r="E4" s="27" t="n"/>
+      <c r="F4" s="27" t="n"/>
+      <c r="G4" s="27" t="n"/>
+      <c r="H4" s="27" t="n"/>
+      <c r="I4" s="27" t="n"/>
+      <c r="J4" s="27" t="n"/>
+      <c r="K4" s="28" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -793,7 +839,7 @@
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>Ferrocons</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
@@ -907,7 +953,7 @@
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>Ferrocons</t>
+          <t>Edificor</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -1155,16 +1201,16 @@
           <t xml:space="preserve">  HOJA 2 — Pastinas</t>
         </is>
       </c>
-      <c r="B13" s="15" t="n"/>
-      <c r="C13" s="15" t="n"/>
-      <c r="D13" s="15" t="n"/>
-      <c r="E13" s="15" t="n"/>
-      <c r="F13" s="15" t="n"/>
-      <c r="G13" s="15" t="n"/>
-      <c r="H13" s="15" t="n"/>
-      <c r="I13" s="15" t="n"/>
-      <c r="J13" s="15" t="n"/>
-      <c r="K13" s="15" t="n"/>
+      <c r="B13" s="27" t="n"/>
+      <c r="C13" s="27" t="n"/>
+      <c r="D13" s="27" t="n"/>
+      <c r="E13" s="27" t="n"/>
+      <c r="F13" s="27" t="n"/>
+      <c r="G13" s="27" t="n"/>
+      <c r="H13" s="27" t="n"/>
+      <c r="I13" s="27" t="n"/>
+      <c r="J13" s="27" t="n"/>
+      <c r="K13" s="28" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
@@ -1343,16 +1389,16 @@
           <t xml:space="preserve">  HOJA 2 — Sanitarios Ferrum Bari</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n"/>
-      <c r="C17" s="17" t="n"/>
-      <c r="D17" s="17" t="n"/>
-      <c r="E17" s="17" t="n"/>
-      <c r="F17" s="17" t="n"/>
-      <c r="G17" s="17" t="n"/>
-      <c r="H17" s="17" t="n"/>
-      <c r="I17" s="17" t="n"/>
-      <c r="J17" s="17" t="n"/>
-      <c r="K17" s="17" t="n"/>
+      <c r="B17" s="27" t="n"/>
+      <c r="C17" s="27" t="n"/>
+      <c r="D17" s="27" t="n"/>
+      <c r="E17" s="27" t="n"/>
+      <c r="F17" s="27" t="n"/>
+      <c r="G17" s="27" t="n"/>
+      <c r="H17" s="27" t="n"/>
+      <c r="I17" s="27" t="n"/>
+      <c r="J17" s="27" t="n"/>
+      <c r="K17" s="28" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
@@ -1588,16 +1634,16 @@
           <t xml:space="preserve">  HOJA 2 — Vanitorys Schneider</t>
         </is>
       </c>
-      <c r="B22" s="15" t="n"/>
-      <c r="C22" s="15" t="n"/>
-      <c r="D22" s="15" t="n"/>
-      <c r="E22" s="15" t="n"/>
-      <c r="F22" s="15" t="n"/>
-      <c r="G22" s="15" t="n"/>
-      <c r="H22" s="15" t="n"/>
-      <c r="I22" s="15" t="n"/>
-      <c r="J22" s="15" t="n"/>
-      <c r="K22" s="15" t="n"/>
+      <c r="B22" s="27" t="n"/>
+      <c r="C22" s="27" t="n"/>
+      <c r="D22" s="27" t="n"/>
+      <c r="E22" s="27" t="n"/>
+      <c r="F22" s="27" t="n"/>
+      <c r="G22" s="27" t="n"/>
+      <c r="H22" s="27" t="n"/>
+      <c r="I22" s="27" t="n"/>
+      <c r="J22" s="27" t="n"/>
+      <c r="K22" s="28" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
@@ -1719,16 +1765,16 @@
           <t xml:space="preserve">  HOJA 2 — Bañera y Desagüe FV</t>
         </is>
       </c>
-      <c r="B25" s="15" t="n"/>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="15" t="n"/>
-      <c r="F25" s="15" t="n"/>
-      <c r="G25" s="15" t="n"/>
-      <c r="H25" s="15" t="n"/>
-      <c r="I25" s="15" t="n"/>
-      <c r="J25" s="15" t="n"/>
-      <c r="K25" s="15" t="n"/>
+      <c r="B25" s="27" t="n"/>
+      <c r="C25" s="27" t="n"/>
+      <c r="D25" s="27" t="n"/>
+      <c r="E25" s="27" t="n"/>
+      <c r="F25" s="27" t="n"/>
+      <c r="G25" s="27" t="n"/>
+      <c r="H25" s="27" t="n"/>
+      <c r="I25" s="27" t="n"/>
+      <c r="J25" s="27" t="n"/>
+      <c r="K25" s="28" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
@@ -1830,7 +1876,7 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>Gili y Cía</t>
+          <t>Barugel</t>
         </is>
       </c>
       <c r="J27" s="8" t="inlineStr">
@@ -1850,16 +1896,16 @@
           <t xml:space="preserve">  HOJA 3 — Grifería FV Mauna</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="5" t="n"/>
-      <c r="K28" s="5" t="n"/>
+      <c r="B28" s="27" t="n"/>
+      <c r="C28" s="27" t="n"/>
+      <c r="D28" s="27" t="n"/>
+      <c r="E28" s="27" t="n"/>
+      <c r="F28" s="27" t="n"/>
+      <c r="G28" s="27" t="n"/>
+      <c r="H28" s="27" t="n"/>
+      <c r="I28" s="27" t="n"/>
+      <c r="J28" s="27" t="n"/>
+      <c r="K28" s="28" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
@@ -1904,7 +1950,7 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>NIMAT</t>
+          <t>Resta</t>
         </is>
       </c>
       <c r="J29" s="8" t="inlineStr">
@@ -1961,7 +2007,7 @@
       </c>
       <c r="I30" s="10" t="inlineStr">
         <is>
-          <t>NIMAT</t>
+          <t>Resta</t>
         </is>
       </c>
       <c r="J30" s="8" t="inlineStr">
@@ -2018,7 +2064,7 @@
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>NIMAT ⭐</t>
+          <t>Resta ⭐</t>
         </is>
       </c>
       <c r="J31" s="8" t="inlineStr">
@@ -2095,16 +2141,16 @@
           <t xml:space="preserve">  HOJA 3 — Accesorios FV</t>
         </is>
       </c>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="5" t="n"/>
-      <c r="I33" s="5" t="n"/>
-      <c r="J33" s="5" t="n"/>
-      <c r="K33" s="5" t="n"/>
+      <c r="B33" s="27" t="n"/>
+      <c r="C33" s="27" t="n"/>
+      <c r="D33" s="27" t="n"/>
+      <c r="E33" s="27" t="n"/>
+      <c r="F33" s="27" t="n"/>
+      <c r="G33" s="27" t="n"/>
+      <c r="H33" s="27" t="n"/>
+      <c r="I33" s="27" t="n"/>
+      <c r="J33" s="27" t="n"/>
+      <c r="K33" s="28" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
@@ -2283,16 +2329,16 @@
           <t xml:space="preserve">  HOJA 4 — Espejos</t>
         </is>
       </c>
-      <c r="B37" s="19" t="n"/>
-      <c r="C37" s="19" t="n"/>
-      <c r="D37" s="19" t="n"/>
-      <c r="E37" s="19" t="n"/>
-      <c r="F37" s="19" t="n"/>
-      <c r="G37" s="19" t="n"/>
-      <c r="H37" s="19" t="n"/>
-      <c r="I37" s="19" t="n"/>
-      <c r="J37" s="19" t="n"/>
-      <c r="K37" s="19" t="n"/>
+      <c r="B37" s="27" t="n"/>
+      <c r="C37" s="27" t="n"/>
+      <c r="D37" s="27" t="n"/>
+      <c r="E37" s="27" t="n"/>
+      <c r="F37" s="27" t="n"/>
+      <c r="G37" s="27" t="n"/>
+      <c r="H37" s="27" t="n"/>
+      <c r="I37" s="27" t="n"/>
+      <c r="J37" s="27" t="n"/>
+      <c r="K37" s="28" t="n"/>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
@@ -2414,16 +2460,16 @@
           <t xml:space="preserve">  HOJA 4 — Roca GAP y Zesty</t>
         </is>
       </c>
-      <c r="B40" s="19" t="n"/>
-      <c r="C40" s="19" t="n"/>
-      <c r="D40" s="19" t="n"/>
-      <c r="E40" s="19" t="n"/>
-      <c r="F40" s="19" t="n"/>
-      <c r="G40" s="19" t="n"/>
-      <c r="H40" s="19" t="n"/>
-      <c r="I40" s="19" t="n"/>
-      <c r="J40" s="19" t="n"/>
-      <c r="K40" s="19" t="n"/>
+      <c r="B40" s="27" t="n"/>
+      <c r="C40" s="27" t="n"/>
+      <c r="D40" s="27" t="n"/>
+      <c r="E40" s="27" t="n"/>
+      <c r="F40" s="27" t="n"/>
+      <c r="G40" s="27" t="n"/>
+      <c r="H40" s="27" t="n"/>
+      <c r="I40" s="27" t="n"/>
+      <c r="J40" s="27" t="n"/>
+      <c r="K40" s="28" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
@@ -2639,7 +2685,7 @@
       </c>
       <c r="I44" s="12" t="inlineStr">
         <is>
-          <t>Remateriales ⭐</t>
+          <t>Resta</t>
         </is>
       </c>
       <c r="J44" s="8" t="inlineStr">
@@ -2735,7 +2781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3207,190 +3253,118 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>NIMAT</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>ventas@nimat.com.ar</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>El Amigo</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>ventas@elamigo.com.ar</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>Grifería FV Mauna</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Sanitarios Ferrum</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t>CABA</t>
         </is>
       </c>
       <c r="G15" s="21" t="inlineStr">
         <is>
-          <t>✅ Mejor ducha Mauna</t>
+          <t>✅ Mejor Ferrum Bari</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>El Amigo</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>ventas@elamigo.com.ar</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Merlino</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>ventas@merlino.com.ar</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>Sanitarios Ferrum</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Vanitory, muebles baño</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>CABA</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>✅ Mejor Ferrum Bari</t>
+          <t>✅ Mejor V. Rivo</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Merlino</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>ventas@merlino.com.ar</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Edificor</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>ventas@edificor.com.ar</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Vanitory, muebles baño</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Revest. porcelánicos</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
         <is>
           <t>CABA</t>
         </is>
       </c>
       <c r="G17" s="21" t="inlineStr">
         <is>
-          <t>✅ Mejor V. Rivo</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Edificor</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>ventas@edificor.com.ar</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>Revest. porcelánicos</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>CABA</t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="inlineStr">
-        <is>
           <t>✅ Mejor Pinto Vivant</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Ferrocons</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>ventas@ferrocons.com.ar</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>Revestimientos</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>CABA</t>
-        </is>
-      </c>
-      <c r="G19" s="21" t="inlineStr">
-        <is>
-          <t>✅ Buen precio Nord Ris</t>
-        </is>
-      </c>
-    </row>
+    <row r="18" ht="22" customHeight="1"/>
+    <row r="19" ht="22" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>

</xml_diff>